<commit_message>
SEM Update on September 18, 2026
</commit_message>
<xml_diff>
--- a/static/data/source/state_and_local_public_education_employment.xlsx
+++ b/static/data/source/state_and_local_public_education_employment.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FT56"/>
+  <dimension ref="A4:FU56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -1254,6 +1254,11 @@
           <t>07/01/2026</t>
         </is>
       </c>
+      <c r="FU4" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1781,10 +1786,13 @@
         <v>11100.7</v>
       </c>
       <c r="FS5">
-        <v>10454.8</v>
+        <v>10452.6</v>
       </c>
       <c r="FT5">
-        <v>9328.6</v>
+        <v>9355</v>
+      </c>
+      <c r="FU5">
+        <v>9750.3</v>
       </c>
     </row>
     <row r="6">
@@ -2316,7 +2324,10 @@
         <v>182.6</v>
       </c>
       <c r="FT6">
-        <v>172</v>
+        <v>172.2</v>
+      </c>
+      <c r="FU6">
+        <v>177.3</v>
       </c>
     </row>
     <row r="7">
@@ -2848,7 +2859,10 @@
         <v>22.1</v>
       </c>
       <c r="FT7">
-        <v>18.5</v>
+        <v>18.4</v>
+      </c>
+      <c r="FU7">
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -3382,6 +3396,9 @@
       <c r="FT8">
         <v>147.6</v>
       </c>
+      <c r="FU8">
+        <v>173.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3914,6 +3931,9 @@
       <c r="FT9">
         <v>78.4</v>
       </c>
+      <c r="FU9">
+        <v>84.9</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4444,7 +4464,10 @@
         <v>1265.6</v>
       </c>
       <c r="FT10">
-        <v>1102.4</v>
+        <v>1093.1</v>
+      </c>
+      <c r="FU10">
+        <v>1160.2</v>
       </c>
     </row>
     <row r="11">
@@ -4978,6 +5001,9 @@
       <c r="FT11">
         <v>215.3</v>
       </c>
+      <c r="FU11">
+        <v>221.2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5510,6 +5536,9 @@
       <c r="FT12">
         <v>98</v>
       </c>
+      <c r="FU12">
+        <v>99.5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6040,7 +6069,10 @@
         <v>36.3</v>
       </c>
       <c r="FT13">
-        <v>34.5</v>
+        <v>34.7</v>
+      </c>
+      <c r="FU13">
+        <v>33.8</v>
       </c>
     </row>
     <row r="14">
@@ -6574,6 +6606,9 @@
       <c r="FT14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FU14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7106,6 +7141,9 @@
       <c r="FT15">
         <v>396</v>
       </c>
+      <c r="FU15">
+        <v>463.3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7636,7 +7674,10 @@
         <v>336.2</v>
       </c>
       <c r="FT16">
-        <v>322</v>
+        <v>323.1</v>
+      </c>
+      <c r="FU16">
+        <v>348.6</v>
       </c>
     </row>
     <row r="17">
@@ -8170,6 +8211,9 @@
       <c r="FT17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FU17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8700,7 +8744,10 @@
         <v>58.3</v>
       </c>
       <c r="FT18">
-        <v>52.9</v>
+        <v>52.4</v>
+      </c>
+      <c r="FU18">
+        <v>53.2</v>
       </c>
     </row>
     <row r="19">
@@ -9232,7 +9279,10 @@
         <v>429.2</v>
       </c>
       <c r="FT19">
-        <v>399.8</v>
+        <v>399.7</v>
+      </c>
+      <c r="FU19">
+        <v>408</v>
       </c>
     </row>
     <row r="20">
@@ -9766,6 +9816,9 @@
       <c r="FT20">
         <v>165.4</v>
       </c>
+      <c r="FU20">
+        <v>204.1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -10296,7 +10349,10 @@
         <v>136.5</v>
       </c>
       <c r="FT21">
-        <v>115.9</v>
+        <v>116.9</v>
+      </c>
+      <c r="FU21">
+        <v>122</v>
       </c>
     </row>
     <row r="22">
@@ -10830,6 +10886,9 @@
       <c r="FT22">
         <v>99.9</v>
       </c>
+      <c r="FU22">
+        <v>106.5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11362,6 +11421,9 @@
       <c r="FT23">
         <v>129.9</v>
       </c>
+      <c r="FU23">
+        <v>152.7</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11894,6 +11956,9 @@
       <c r="FT24">
         <v>133.3</v>
       </c>
+      <c r="FU24">
+        <v>140.5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12424,7 +12489,10 @@
         <v>47.1</v>
       </c>
       <c r="FT25">
-        <v>40.2</v>
+        <v>39.2</v>
+      </c>
+      <c r="FU25">
+        <v>38.7</v>
       </c>
     </row>
     <row r="26">
@@ -12958,6 +13026,9 @@
       <c r="FT26">
         <v>201.2</v>
       </c>
+      <c r="FU26">
+        <v>201.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13490,6 +13561,9 @@
       <c r="FT27">
         <v>217.7</v>
       </c>
+      <c r="FU27">
+        <v>215</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -14022,6 +14096,9 @@
       <c r="FT28">
         <v>275.7</v>
       </c>
+      <c r="FU28">
+        <v>280.7</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14552,7 +14629,10 @@
         <v>205.5</v>
       </c>
       <c r="FT29">
-        <v>173.5</v>
+        <v>173.7</v>
+      </c>
+      <c r="FU29">
+        <v>169.9</v>
       </c>
     </row>
     <row r="30">
@@ -15084,7 +15164,10 @@
         <v>98.8</v>
       </c>
       <c r="FT30">
-        <v>93.1</v>
+        <v>95</v>
+      </c>
+      <c r="FU30">
+        <v>99.6</v>
       </c>
     </row>
     <row r="31">
@@ -15618,6 +15701,9 @@
       <c r="FT31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FU31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -16150,6 +16236,9 @@
       <c r="FT32">
         <v>34.8</v>
       </c>
+      <c r="FU32">
+        <v>36</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -16682,6 +16771,9 @@
       <c r="FT33">
         <v>80.4</v>
       </c>
+      <c r="FU33">
+        <v>81.8</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -17214,6 +17306,9 @@
       <c r="FT34">
         <v>72.5</v>
       </c>
+      <c r="FU34">
+        <v>76.9</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -17744,7 +17839,10 @@
         <v>39.8</v>
       </c>
       <c r="FT35">
-        <v>32.5</v>
+        <v>32.1</v>
+      </c>
+      <c r="FU35">
+        <v>32.6</v>
       </c>
     </row>
     <row r="36">
@@ -18278,6 +18376,9 @@
       <c r="FT36">
         <v>266.7</v>
       </c>
+      <c r="FU36">
+        <v>262.7</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -18808,7 +18909,10 @@
         <v>70.9</v>
       </c>
       <c r="FT37">
-        <v>62.8</v>
+        <v>64.5</v>
+      </c>
+      <c r="FU37">
+        <v>74.3</v>
       </c>
     </row>
     <row r="38">
@@ -19340,7 +19444,10 @@
         <v>695.9</v>
       </c>
       <c r="FT38">
-        <v>580</v>
+        <v>581.8</v>
+      </c>
+      <c r="FU38">
+        <v>574.6</v>
       </c>
     </row>
     <row r="39">
@@ -19874,6 +19981,9 @@
       <c r="FT39">
         <v>262.7</v>
       </c>
+      <c r="FU39">
+        <v>307.9</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -20406,6 +20516,9 @@
       <c r="FT40">
         <v>29.5</v>
       </c>
+      <c r="FU40">
+        <v>30.1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -20936,7 +21049,10 @@
         <v>361.2</v>
       </c>
       <c r="FT41">
-        <v>347.1</v>
+        <v>348.1</v>
+      </c>
+      <c r="FU41">
+        <v>353.4</v>
       </c>
     </row>
     <row r="42">
@@ -21470,6 +21586,9 @@
       <c r="FT42">
         <v>132.6</v>
       </c>
+      <c r="FU42">
+        <v>138.5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -22000,7 +22119,10 @@
         <v>136.3</v>
       </c>
       <c r="FT43">
-        <v>105.7</v>
+        <v>106.2</v>
+      </c>
+      <c r="FU43">
+        <v>108.5</v>
       </c>
     </row>
     <row r="44">
@@ -22534,6 +22656,9 @@
       <c r="FT44">
         <v>279</v>
       </c>
+      <c r="FU44">
+        <v>286.9</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -23066,6 +23191,9 @@
       <c r="FT45">
         <v>22.9</v>
       </c>
+      <c r="FU45">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -23596,7 +23724,10 @@
         <v>167.7</v>
       </c>
       <c r="FT46">
-        <v>160.3</v>
+        <v>158.9</v>
+      </c>
+      <c r="FU46">
+        <v>164.6</v>
       </c>
     </row>
     <row r="47">
@@ -24128,7 +24259,10 @@
         <v>34</v>
       </c>
       <c r="FT47">
-        <v>28.2</v>
+        <v>28.3</v>
+      </c>
+      <c r="FU47">
+        <v>29.5</v>
       </c>
     </row>
     <row r="48">
@@ -24662,6 +24796,9 @@
       <c r="FT48">
         <v>178.2</v>
       </c>
+      <c r="FU48">
+        <v>192.8</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -25192,7 +25329,10 @@
         <v>1162.2</v>
       </c>
       <c r="FT49">
-        <v>1081.8</v>
+        <v>1084.7</v>
+      </c>
+      <c r="FU49">
+        <v>1115.8</v>
       </c>
     </row>
     <row r="50">
@@ -25726,6 +25866,9 @@
       <c r="FT50">
         <v>111</v>
       </c>
+      <c r="FU50">
+        <v>119.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -26256,7 +26399,10 @@
         <v>29.2</v>
       </c>
       <c r="FT51">
-        <v>25.5</v>
+        <v>25.8</v>
+      </c>
+      <c r="FU51">
+        <v>25</v>
       </c>
     </row>
     <row r="52">
@@ -26788,7 +26934,10 @@
         <v>337</v>
       </c>
       <c r="FT52">
-        <v>298.8</v>
+        <v>299.6</v>
+      </c>
+      <c r="FU52">
+        <v>308.7</v>
       </c>
     </row>
     <row r="53">
@@ -27322,6 +27471,9 @@
       <c r="FT53">
         <v>236.8</v>
       </c>
+      <c r="FU53">
+        <v>226.6</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -27854,6 +28006,9 @@
       <c r="FT54">
         <v>54</v>
       </c>
+      <c r="FU54">
+        <v>55.9</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -28384,7 +28539,10 @@
         <v>184.9</v>
       </c>
       <c r="FT55">
-        <v>170.7</v>
+        <v>170.4</v>
+      </c>
+      <c r="FU55">
+        <v>168.4</v>
       </c>
     </row>
     <row r="56">
@@ -28916,7 +29074,10 @@
         <v>27.9</v>
       </c>
       <c r="FT56">
-        <v>24.5</v>
+        <v>24.4</v>
+      </c>
+      <c r="FU56">
+        <v>24.9</v>
       </c>
     </row>
   </sheetData>
@@ -28928,7 +29089,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FH56"/>
+  <dimension ref="A4:FI56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -29752,6 +29913,11 @@
           <t>07/01/2026</t>
         </is>
       </c>
+      <c r="FI4" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -30243,10 +30409,13 @@
         <v>-0.00900762946215444</v>
       </c>
       <c r="FG5">
-        <v>-0.469340543216469</v>
+        <v>-0.490284745956358</v>
       </c>
       <c r="FH5">
-        <v>-0.565995501881326</v>
+        <v>-0.284596608290616</v>
+      </c>
+      <c r="FI5">
+        <v>-0.594376363599283</v>
       </c>
     </row>
     <row r="6">
@@ -30742,7 +30911,10 @@
         <v>3.28054298642535</v>
       </c>
       <c r="FH6">
-        <v>2.9940119760479</v>
+        <v>3.11377245508981</v>
+      </c>
+      <c r="FI6">
+        <v>2.96167247386761</v>
       </c>
     </row>
     <row r="7">
@@ -31238,7 +31410,10 @@
         <v>-3.07017543859649</v>
       </c>
       <c r="FH7">
-        <v>-1.06951871657756</v>
+        <v>-1.60427807486633</v>
+      </c>
+      <c r="FI7">
+        <v>-1.78571428571428</v>
       </c>
     </row>
     <row r="8">
@@ -31736,6 +31911,9 @@
       <c r="FH8">
         <v>-0.873069173942232</v>
       </c>
+      <c r="FI8">
+        <v>-0.913763563677911</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -32232,6 +32410,9 @@
       <c r="FH9">
         <v>-0.633713561470215</v>
       </c>
+      <c r="FI9">
+        <v>-0.817757009345781</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -32726,7 +32907,10 @@
         <v>-2.14180777855098</v>
       </c>
       <c r="FH10">
-        <v>-0.675736552842578</v>
+        <v>-1.51364987836742</v>
+      </c>
+      <c r="FI10">
+        <v>2.54551882623298</v>
       </c>
     </row>
     <row r="11">
@@ -33224,6 +33408,9 @@
       <c r="FH11">
         <v>1.60453043888626</v>
       </c>
+      <c r="FI11">
+        <v>0.682749203459263</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -33720,6 +33907,9 @@
       <c r="FH12">
         <v>-0.709219858156017</v>
       </c>
+      <c r="FI12">
+        <v>-0.896414342629488</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -34214,7 +34404,10 @@
         <v>-2.15633423180592</v>
       </c>
       <c r="FH13">
-        <v>-1.70940170940171</v>
+        <v>-1.13960113960114</v>
+      </c>
+      <c r="FI13">
+        <v>-2.02898550724638</v>
       </c>
     </row>
     <row r="14">
@@ -34712,6 +34905,9 @@
       <c r="FH14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FI14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -35208,6 +35404,9 @@
       <c r="FH15">
         <v>-1.36986301369863</v>
       </c>
+      <c r="FI15">
+        <v>-1.19428449562806</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -35702,7 +35901,10 @@
         <v>0.478182904961154</v>
       </c>
       <c r="FH16">
-        <v>1.13065326633167</v>
+        <v>1.47613065326635</v>
+      </c>
+      <c r="FI16">
+        <v>1.6326530612245</v>
       </c>
     </row>
     <row r="17">
@@ -36200,6 +36402,9 @@
       <c r="FH17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FI17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -36694,7 +36899,10 @@
         <v>-2.34505862646566</v>
       </c>
       <c r="FH18">
-        <v>-1.85528756957328</v>
+        <v>-2.78293135435993</v>
+      </c>
+      <c r="FI18">
+        <v>-3.79746835443037</v>
       </c>
     </row>
     <row r="19">
@@ -37190,7 +37398,10 @@
         <v>-0.139599813866894</v>
       </c>
       <c r="FH19">
-        <v>1.11279716742539</v>
+        <v>1.08750632271118</v>
+      </c>
+      <c r="FI19">
+        <v>0.29498525073746</v>
       </c>
     </row>
     <row r="20">
@@ -37688,6 +37899,9 @@
       <c r="FH20">
         <v>-5.48571428571428</v>
       </c>
+      <c r="FI20">
+        <v>-8.39317773788152</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -38182,7 +38396,10 @@
         <v>-0.146305779078265</v>
       </c>
       <c r="FH21">
-        <v>1.0462074978204</v>
+        <v>1.9180470793374</v>
+      </c>
+      <c r="FI21">
+        <v>1.66666666666667</v>
       </c>
     </row>
     <row r="22">
@@ -38680,6 +38897,9 @@
       <c r="FH22">
         <v>0.200601805416237</v>
       </c>
+      <c r="FI22">
+        <v>0.188146754468475</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -39176,6 +39396,9 @@
       <c r="FH23">
         <v>-0.612088752869153</v>
       </c>
+      <c r="FI23">
+        <v>-0.391389432485338</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -39672,6 +39895,9 @@
       <c r="FH24">
         <v>-0.0749625187406041</v>
       </c>
+      <c r="FI24">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -40166,7 +40392,10 @@
         <v>-3.08641975308642</v>
       </c>
       <c r="FH25">
-        <v>3.87596899224806</v>
+        <v>1.29198966408269</v>
+      </c>
+      <c r="FI25">
+        <v>0.259067357512957</v>
       </c>
     </row>
     <row r="26">
@@ -40664,6 +40893,9 @@
       <c r="FH26">
         <v>1.00401606425701</v>
       </c>
+      <c r="FI26">
+        <v>0.849575212393797</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -41160,6 +41392,9 @@
       <c r="FH27">
         <v>0.184077312471227</v>
       </c>
+      <c r="FI27">
+        <v>0.233100233100233</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -41656,6 +41891,9 @@
       <c r="FH28">
         <v>3.25842696629215</v>
       </c>
+      <c r="FI28">
+        <v>3.1985294117647</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -42150,7 +42388,10 @@
         <v>0.784698381559585</v>
       </c>
       <c r="FH29">
-        <v>1.46198830409357</v>
+        <v>1.57894736842105</v>
+      </c>
+      <c r="FI29">
+        <v>1.55409444112371</v>
       </c>
     </row>
     <row r="30">
@@ -42646,7 +42887,10 @@
         <v>1.33333333333335</v>
       </c>
       <c r="FH30">
-        <v>2.42024202420242</v>
+        <v>4.5104510451045</v>
+      </c>
+      <c r="FI30">
+        <v>1.32248219735505</v>
       </c>
     </row>
     <row r="31">
@@ -43144,6 +43388,9 @@
       <c r="FH31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FI31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -43640,6 +43887,9 @@
       <c r="FH32">
         <v>-1.41643059490085</v>
       </c>
+      <c r="FI32">
+        <v>-1.63934426229509</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -44136,6 +44386,9 @@
       <c r="FH33">
         <v>0.124533001245341</v>
       </c>
+      <c r="FI33">
+        <v>-0.365408038976854</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -44632,6 +44885,9 @@
       <c r="FH34">
         <v>0.554785020804446</v>
       </c>
+      <c r="FI34">
+        <v>0.260756192959586</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -45126,7 +45382,10 @@
         <v>1.01522842639595</v>
       </c>
       <c r="FH35">
-        <v>3.17460317460317</v>
+        <v>1.90476190476191</v>
+      </c>
+      <c r="FI35">
+        <v>1.55763239875389</v>
       </c>
     </row>
     <row r="36">
@@ -45624,6 +45883,9 @@
       <c r="FH36">
         <v>0.489826676714398</v>
       </c>
+      <c r="FI36">
+        <v>0.458891013384317</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -46118,7 +46380,10 @@
         <v>-1.25348189415041</v>
       </c>
       <c r="FH37">
-        <v>0.641025641025639</v>
+        <v>3.36538461538462</v>
+      </c>
+      <c r="FI37">
+        <v>5.09193776520508</v>
       </c>
     </row>
     <row r="38">
@@ -46614,7 +46879,10 @@
         <v>1.72489402134192</v>
       </c>
       <c r="FH38">
-        <v>2.43730130695866</v>
+        <v>2.7552101730837</v>
+      </c>
+      <c r="FI38">
+        <v>2.84589224986576</v>
       </c>
     </row>
     <row r="39">
@@ -47112,6 +47380,9 @@
       <c r="FH39">
         <v>0.0380807311500251</v>
       </c>
+      <c r="FI39">
+        <v>0.0649983750406203</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -47608,6 +47879,9 @@
       <c r="FH40">
         <v>0.340136054421774</v>
       </c>
+      <c r="FI40">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -48102,7 +48376,10 @@
         <v>0.305470702582622</v>
       </c>
       <c r="FH41">
-        <v>-0.800228636753345</v>
+        <v>-0.514432695055717</v>
+      </c>
+      <c r="FI41">
+        <v>0.113314447592062</v>
       </c>
     </row>
     <row r="42">
@@ -48600,6 +48877,9 @@
       <c r="FH42">
         <v>1.45371078806427</v>
       </c>
+      <c r="FI42">
+        <v>1.46520146520147</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -49094,7 +49374,10 @@
         <v>-2.98932384341636</v>
       </c>
       <c r="FH43">
-        <v>-2.93847566574838</v>
+        <v>-2.4793388429752</v>
+      </c>
+      <c r="FI43">
+        <v>-2.60323159784559</v>
       </c>
     </row>
     <row r="44">
@@ -49592,6 +49875,9 @@
       <c r="FH44">
         <v>0.758396533044429</v>
       </c>
+      <c r="FI44">
+        <v>0.702000702000702</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -50088,6 +50374,9 @@
       <c r="FH45">
         <v>-1.7167381974249</v>
       </c>
+      <c r="FI45">
+        <v>-1.7391304347826</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -50582,7 +50871,10 @@
         <v>0.841852074564027</v>
       </c>
       <c r="FH46">
-        <v>1.84243964421857</v>
+        <v>0.952986022871683</v>
+      </c>
+      <c r="FI46">
+        <v>-1.08173076923078</v>
       </c>
     </row>
     <row r="47">
@@ -51078,7 +51370,10 @@
         <v>-2.01729106628243</v>
       </c>
       <c r="FH47">
-        <v>-1.39860139860141</v>
+        <v>-1.04895104895105</v>
+      </c>
+      <c r="FI47">
+        <v>-1.00671140939598</v>
       </c>
     </row>
     <row r="48">
@@ -51576,6 +51871,9 @@
       <c r="FH48">
         <v>2.23752151462994</v>
       </c>
+      <c r="FI48">
+        <v>2.28116710875332</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -52070,7 +52368,10 @@
         <v>0.0430403718688129</v>
       </c>
       <c r="FH49">
-        <v>-0.110803324099727</v>
+        <v>0.156971375807945</v>
+      </c>
+      <c r="FI49">
+        <v>0.585955106824123</v>
       </c>
     </row>
     <row r="50">
@@ -52568,6 +52869,9 @@
       <c r="FH50">
         <v>-2.80210157618214</v>
       </c>
+      <c r="FI50">
+        <v>-1.56249999999999</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -53062,7 +53366,10 @@
         <v>-1.35135135135135</v>
       </c>
       <c r="FH51">
-        <v>6.25</v>
+        <v>7.49999999999999</v>
+      </c>
+      <c r="FI51">
+        <v>-3.47490347490347</v>
       </c>
     </row>
     <row r="52">
@@ -53558,7 +53865,10 @@
         <v>2.86935286935286</v>
       </c>
       <c r="FH52">
-        <v>1.66723375297721</v>
+        <v>1.93943518203472</v>
+      </c>
+      <c r="FI52">
+        <v>1.84757505773671</v>
       </c>
     </row>
     <row r="53">
@@ -54056,6 +54366,9 @@
       <c r="FH53">
         <v>-2.99057763211798</v>
       </c>
+      <c r="FI53">
+        <v>-2.24331320103538</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -54552,6 +54865,9 @@
       <c r="FH54">
         <v>3.44827586206896</v>
       </c>
+      <c r="FI54">
+        <v>2.75735294117647</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -55046,7 +55362,10 @@
         <v>-2.63296471827276</v>
       </c>
       <c r="FH55">
-        <v>-1.1008111239861</v>
+        <v>-1.27462340672075</v>
+      </c>
+      <c r="FI55">
+        <v>-3.77142857142858</v>
       </c>
     </row>
     <row r="56">
@@ -55542,7 +55861,10 @@
         <v>-3.12500000000001</v>
       </c>
       <c r="FH56">
-        <v>-3.92156862745098</v>
+        <v>-4.31372549019608</v>
+      </c>
+      <c r="FI56">
+        <v>-3.48837209302325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SEM update on October 21, 2026
</commit_message>
<xml_diff>
--- a/static/data/source/state_and_local_public_education_employment.xlsx
+++ b/static/data/source/state_and_local_public_education_employment.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FU56"/>
+  <dimension ref="A4:FV56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -1259,6 +1259,11 @@
           <t>08/01/2026</t>
         </is>
       </c>
+      <c r="FV4" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1789,10 +1794,13 @@
         <v>10452.6</v>
       </c>
       <c r="FT5">
-        <v>9355</v>
+        <v>9355.9</v>
       </c>
       <c r="FU5">
-        <v>9750.3</v>
+        <v>9770.4</v>
+      </c>
+      <c r="FV5">
+        <v>10843</v>
       </c>
     </row>
     <row r="6">
@@ -2327,7 +2335,10 @@
         <v>172.2</v>
       </c>
       <c r="FU6">
-        <v>177.3</v>
+        <v>177.2</v>
+      </c>
+      <c r="FV6">
+        <v>184.2</v>
       </c>
     </row>
     <row r="7">
@@ -2862,7 +2873,10 @@
         <v>18.4</v>
       </c>
       <c r="FU7">
-        <v>22</v>
+        <v>21.8</v>
+      </c>
+      <c r="FV7">
+        <v>25.4</v>
       </c>
     </row>
     <row r="8">
@@ -3397,7 +3411,10 @@
         <v>147.6</v>
       </c>
       <c r="FU8">
-        <v>173.5</v>
+        <v>174.8</v>
+      </c>
+      <c r="FV8">
+        <v>197.9</v>
       </c>
     </row>
     <row r="9">
@@ -3934,6 +3951,9 @@
       <c r="FU9">
         <v>84.9</v>
       </c>
+      <c r="FV9">
+        <v>96</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4467,7 +4487,10 @@
         <v>1093.1</v>
       </c>
       <c r="FU10">
-        <v>1160.2</v>
+        <v>1163.9</v>
+      </c>
+      <c r="FV10">
+        <v>1229.6</v>
       </c>
     </row>
     <row r="11">
@@ -5002,7 +5025,10 @@
         <v>215.3</v>
       </c>
       <c r="FU11">
-        <v>221.2</v>
+        <v>222.2</v>
+      </c>
+      <c r="FV11">
+        <v>241</v>
       </c>
     </row>
     <row r="12">
@@ -5539,6 +5565,9 @@
       <c r="FU12">
         <v>99.5</v>
       </c>
+      <c r="FV12">
+        <v>121.7</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6072,7 +6101,10 @@
         <v>34.7</v>
       </c>
       <c r="FU13">
-        <v>33.8</v>
+        <v>34</v>
+      </c>
+      <c r="FV13">
+        <v>38.1</v>
       </c>
     </row>
     <row r="14">
@@ -6609,6 +6641,9 @@
       <c r="FU14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FV14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7142,7 +7177,10 @@
         <v>396</v>
       </c>
       <c r="FU15">
-        <v>463.3</v>
+        <v>464</v>
+      </c>
+      <c r="FV15">
+        <v>488.4</v>
       </c>
     </row>
     <row r="16">
@@ -7677,7 +7715,10 @@
         <v>323.1</v>
       </c>
       <c r="FU16">
-        <v>348.6</v>
+        <v>346.7</v>
+      </c>
+      <c r="FV16">
+        <v>355.8</v>
       </c>
     </row>
     <row r="17">
@@ -8214,6 +8255,9 @@
       <c r="FU17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FV17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8747,7 +8791,10 @@
         <v>52.4</v>
       </c>
       <c r="FU18">
-        <v>53.2</v>
+        <v>53.1</v>
+      </c>
+      <c r="FV18">
+        <v>58.8</v>
       </c>
     </row>
     <row r="19">
@@ -9282,7 +9329,10 @@
         <v>399.7</v>
       </c>
       <c r="FU19">
-        <v>408</v>
+        <v>407.9</v>
+      </c>
+      <c r="FV19">
+        <v>456.2</v>
       </c>
     </row>
     <row r="20">
@@ -9817,7 +9867,10 @@
         <v>165.4</v>
       </c>
       <c r="FU20">
-        <v>204.1</v>
+        <v>203.9</v>
+      </c>
+      <c r="FV20">
+        <v>212.4</v>
       </c>
     </row>
     <row r="21">
@@ -10354,6 +10407,9 @@
       <c r="FU21">
         <v>122</v>
       </c>
+      <c r="FV21">
+        <v>148.4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -10889,6 +10945,9 @@
       <c r="FU22">
         <v>106.5</v>
       </c>
+      <c r="FV22">
+        <v>135.1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11424,6 +11483,9 @@
       <c r="FU23">
         <v>152.7</v>
       </c>
+      <c r="FV23">
+        <v>162.3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11959,6 +12021,9 @@
       <c r="FU24">
         <v>140.5</v>
       </c>
+      <c r="FV24">
+        <v>150.5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12494,6 +12559,9 @@
       <c r="FU25">
         <v>38.7</v>
       </c>
+      <c r="FV25">
+        <v>47.7</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13029,6 +13097,9 @@
       <c r="FU26">
         <v>201.8</v>
       </c>
+      <c r="FV26">
+        <v>222.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13564,6 +13635,9 @@
       <c r="FU27">
         <v>215</v>
       </c>
+      <c r="FV27">
+        <v>241.3</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -14099,6 +14173,9 @@
       <c r="FU28">
         <v>280.7</v>
       </c>
+      <c r="FV28">
+        <v>328.5</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14632,7 +14709,10 @@
         <v>173.7</v>
       </c>
       <c r="FU29">
-        <v>169.9</v>
+        <v>169.7</v>
+      </c>
+      <c r="FV29">
+        <v>200.6</v>
       </c>
     </row>
     <row r="30">
@@ -15167,7 +15247,10 @@
         <v>95</v>
       </c>
       <c r="FU30">
-        <v>99.6</v>
+        <v>99.3</v>
+      </c>
+      <c r="FV30">
+        <v>105.2</v>
       </c>
     </row>
     <row r="31">
@@ -15704,6 +15787,9 @@
       <c r="FU31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FV31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -16239,6 +16325,9 @@
       <c r="FU32">
         <v>36</v>
       </c>
+      <c r="FV32">
+        <v>40.7</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -16772,7 +16861,10 @@
         <v>80.4</v>
       </c>
       <c r="FU33">
-        <v>81.8</v>
+        <v>82</v>
+      </c>
+      <c r="FV33">
+        <v>94.2</v>
       </c>
     </row>
     <row r="34">
@@ -17309,6 +17401,9 @@
       <c r="FU34">
         <v>76.9</v>
       </c>
+      <c r="FV34">
+        <v>88.6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -17844,6 +17939,9 @@
       <c r="FU35">
         <v>32.6</v>
       </c>
+      <c r="FV35">
+        <v>43.8</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -18379,6 +18477,9 @@
       <c r="FU36">
         <v>262.7</v>
       </c>
+      <c r="FV36">
+        <v>312.8</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -18912,7 +19013,10 @@
         <v>64.5</v>
       </c>
       <c r="FU37">
-        <v>74.3</v>
+        <v>73.7</v>
+      </c>
+      <c r="FV37">
+        <v>80.6</v>
       </c>
     </row>
     <row r="38">
@@ -19447,7 +19551,10 @@
         <v>581.8</v>
       </c>
       <c r="FU38">
-        <v>574.6</v>
+        <v>566.3</v>
+      </c>
+      <c r="FV38">
+        <v>664.8</v>
       </c>
     </row>
     <row r="39">
@@ -19984,6 +20091,9 @@
       <c r="FU39">
         <v>307.9</v>
       </c>
+      <c r="FV39">
+        <v>337.5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -20519,6 +20629,9 @@
       <c r="FU40">
         <v>30.1</v>
       </c>
+      <c r="FV40">
+        <v>38.4</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -21052,7 +21165,10 @@
         <v>348.1</v>
       </c>
       <c r="FU41">
-        <v>353.4</v>
+        <v>354.7</v>
+      </c>
+      <c r="FV41">
+        <v>384.1</v>
       </c>
     </row>
     <row r="42">
@@ -21589,6 +21705,9 @@
       <c r="FU42">
         <v>138.5</v>
       </c>
+      <c r="FV42">
+        <v>156.6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -22122,7 +22241,10 @@
         <v>106.2</v>
       </c>
       <c r="FU43">
-        <v>108.5</v>
+        <v>109.6</v>
+      </c>
+      <c r="FV43">
+        <v>125.4</v>
       </c>
     </row>
     <row r="44">
@@ -22659,6 +22781,9 @@
       <c r="FU44">
         <v>286.9</v>
       </c>
+      <c r="FV44">
+        <v>333.3</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -23194,6 +23319,9 @@
       <c r="FU45">
         <v>22.6</v>
       </c>
+      <c r="FV45">
+        <v>28.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -23727,7 +23855,10 @@
         <v>158.9</v>
       </c>
       <c r="FU46">
-        <v>164.6</v>
+        <v>164.8</v>
+      </c>
+      <c r="FV46">
+        <v>174.7</v>
       </c>
     </row>
     <row r="47">
@@ -24264,6 +24395,9 @@
       <c r="FU47">
         <v>29.5</v>
       </c>
+      <c r="FV47">
+        <v>37.4</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -24799,6 +24933,9 @@
       <c r="FU48">
         <v>192.8</v>
       </c>
+      <c r="FV48">
+        <v>220</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -25332,7 +25469,10 @@
         <v>1084.7</v>
       </c>
       <c r="FU49">
-        <v>1115.8</v>
+        <v>1119.4</v>
+      </c>
+      <c r="FV49">
+        <v>1174.2</v>
       </c>
     </row>
     <row r="50">
@@ -25869,6 +26009,9 @@
       <c r="FU50">
         <v>119.7</v>
       </c>
+      <c r="FV50">
+        <v>131.4</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -26402,7 +26545,10 @@
         <v>25.8</v>
       </c>
       <c r="FU51">
-        <v>25</v>
+        <v>25.2</v>
+      </c>
+      <c r="FV51">
+        <v>31.4</v>
       </c>
     </row>
     <row r="52">
@@ -26937,7 +27083,10 @@
         <v>299.6</v>
       </c>
       <c r="FU52">
-        <v>308.7</v>
+        <v>311.5</v>
+      </c>
+      <c r="FV52">
+        <v>345.7</v>
       </c>
     </row>
     <row r="53">
@@ -27472,7 +27621,10 @@
         <v>236.8</v>
       </c>
       <c r="FU53">
-        <v>226.6</v>
+        <v>226.2</v>
+      </c>
+      <c r="FV53">
+        <v>239.2</v>
       </c>
     </row>
     <row r="54">
@@ -28009,6 +28161,9 @@
       <c r="FU54">
         <v>55.9</v>
       </c>
+      <c r="FV54">
+        <v>61.7</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -28542,7 +28697,10 @@
         <v>170.4</v>
       </c>
       <c r="FU55">
-        <v>168.4</v>
+        <v>169.9</v>
+      </c>
+      <c r="FV55">
+        <v>200.2</v>
       </c>
     </row>
     <row r="56">
@@ -29077,7 +29235,10 @@
         <v>24.4</v>
       </c>
       <c r="FU56">
-        <v>24.9</v>
+        <v>25</v>
+      </c>
+      <c r="FV56">
+        <v>29.7</v>
       </c>
     </row>
   </sheetData>
@@ -29089,7 +29250,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FI56"/>
+  <dimension ref="A4:FJ56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -29918,6 +30079,11 @@
           <t>08/01/2026</t>
         </is>
       </c>
+      <c r="FJ4" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -30412,10 +30578,13 @@
         <v>-0.490284745956358</v>
       </c>
       <c r="FH5">
-        <v>-0.284596608290616</v>
+        <v>-0.275003464190937</v>
       </c>
       <c r="FI5">
-        <v>-0.594376363599283</v>
+        <v>-0.389454152478426</v>
+      </c>
+      <c r="FJ5">
+        <v>-0.46449291327018</v>
       </c>
     </row>
     <row r="6">
@@ -30914,7 +31083,10 @@
         <v>3.11377245508981</v>
       </c>
       <c r="FI6">
-        <v>2.96167247386761</v>
+        <v>2.90360046457607</v>
+      </c>
+      <c r="FJ6">
+        <v>2.84757118927973</v>
       </c>
     </row>
     <row r="7">
@@ -31413,7 +31585,10 @@
         <v>-1.60427807486633</v>
       </c>
       <c r="FI7">
-        <v>-1.78571428571428</v>
+        <v>-2.67857142857144</v>
+      </c>
+      <c r="FJ7">
+        <v>-4.15094339622642</v>
       </c>
     </row>
     <row r="8">
@@ -31912,7 +32087,10 @@
         <v>-0.873069173942232</v>
       </c>
       <c r="FI8">
-        <v>-0.913763563677911</v>
+        <v>-0.171330668189612</v>
+      </c>
+      <c r="FJ8">
+        <v>-0.100959111559827</v>
       </c>
     </row>
     <row r="9">
@@ -32413,6 +32591,9 @@
       <c r="FI9">
         <v>-0.817757009345781</v>
       </c>
+      <c r="FJ9">
+        <v>-0.311526479750791</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -32910,7 +33091,10 @@
         <v>-1.51364987836742</v>
       </c>
       <c r="FI10">
-        <v>2.54551882623298</v>
+        <v>2.87254728654764</v>
+      </c>
+      <c r="FJ10">
+        <v>2.40692929124676</v>
       </c>
     </row>
     <row r="11">
@@ -33409,7 +33593,10 @@
         <v>1.60453043888626</v>
       </c>
       <c r="FI11">
-        <v>0.682749203459263</v>
+        <v>1.13791533909877</v>
+      </c>
+      <c r="FJ11">
+        <v>0.752508361204018</v>
       </c>
     </row>
     <row r="12">
@@ -33910,6 +34097,9 @@
       <c r="FI12">
         <v>-0.896414342629488</v>
       </c>
+      <c r="FJ12">
+        <v>-0.734094616639471</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -34407,7 +34597,10 @@
         <v>-1.13960113960114</v>
       </c>
       <c r="FI13">
-        <v>-2.02898550724638</v>
+        <v>-1.44927536231884</v>
+      </c>
+      <c r="FJ13">
+        <v>-1.55038759689923</v>
       </c>
     </row>
     <row r="14">
@@ -34908,6 +35101,9 @@
       <c r="FI14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FJ14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -35405,7 +35601,10 @@
         <v>-1.36986301369863</v>
       </c>
       <c r="FI15">
-        <v>-1.19428449562806</v>
+        <v>-1.04499893367455</v>
+      </c>
+      <c r="FJ15">
+        <v>-1.29345189975747</v>
       </c>
     </row>
     <row r="16">
@@ -35904,7 +36103,10 @@
         <v>1.47613065326635</v>
       </c>
       <c r="FI16">
-        <v>1.6326530612245</v>
+        <v>1.07871720116619</v>
+      </c>
+      <c r="FJ16">
+        <v>1.48317170564747</v>
       </c>
     </row>
     <row r="17">
@@ -36405,6 +36607,9 @@
       <c r="FI17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FJ17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -36902,7 +37107,10 @@
         <v>-2.78293135435993</v>
       </c>
       <c r="FI18">
-        <v>-3.79746835443037</v>
+        <v>-3.97830018083183</v>
+      </c>
+      <c r="FJ18">
+        <v>-3.76432078559739</v>
       </c>
     </row>
     <row r="19">
@@ -37401,7 +37609,10 @@
         <v>1.08750632271118</v>
       </c>
       <c r="FI19">
-        <v>0.29498525073746</v>
+        <v>0.270403146509333</v>
+      </c>
+      <c r="FJ19">
+        <v>-0.218722659667542</v>
       </c>
     </row>
     <row r="20">
@@ -37900,7 +38111,10 @@
         <v>-5.48571428571428</v>
       </c>
       <c r="FI20">
-        <v>-8.39317773788152</v>
+        <v>-8.48294434470377</v>
+      </c>
+      <c r="FJ20">
+        <v>-5.85106382978725</v>
       </c>
     </row>
     <row r="21">
@@ -38401,6 +38615,9 @@
       <c r="FI21">
         <v>1.66666666666667</v>
       </c>
+      <c r="FJ21">
+        <v>2.48618784530386</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -38900,6 +39117,9 @@
       <c r="FI22">
         <v>0.188146754468475</v>
       </c>
+      <c r="FJ22">
+        <v>0.520833333333325</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -39399,6 +39619,9 @@
       <c r="FI23">
         <v>-0.391389432485338</v>
       </c>
+      <c r="FJ23">
+        <v>-0.429447852760729</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -39898,6 +40121,9 @@
       <c r="FI24">
         <v>0</v>
       </c>
+      <c r="FJ24">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -40397,6 +40623,9 @@
       <c r="FI25">
         <v>0.259067357512957</v>
       </c>
+      <c r="FJ25">
+        <v>0.421052631578953</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -40896,6 +41125,9 @@
       <c r="FI26">
         <v>0.849575212393797</v>
       </c>
+      <c r="FJ26">
+        <v>0.632339656729903</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -41395,6 +41627,9 @@
       <c r="FI27">
         <v>0.233100233100233</v>
       </c>
+      <c r="FJ27">
+        <v>0.166044001660442</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -41894,6 +42129,9 @@
       <c r="FI28">
         <v>3.1985294117647</v>
       </c>
+      <c r="FJ28">
+        <v>2.75258054426025</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -42391,7 +42629,10 @@
         <v>1.57894736842105</v>
       </c>
       <c r="FI29">
-        <v>1.55409444112371</v>
+        <v>1.43454871488343</v>
+      </c>
+      <c r="FJ29">
+        <v>-0.545364402578083</v>
       </c>
     </row>
     <row r="30">
@@ -42890,7 +43131,10 @@
         <v>4.5104510451045</v>
       </c>
       <c r="FI30">
-        <v>1.32248219735505</v>
+        <v>1.01729399796541</v>
+      </c>
+      <c r="FJ30">
+        <v>1.0566762728146</v>
       </c>
     </row>
     <row r="31">
@@ -43391,6 +43635,9 @@
       <c r="FI31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FJ31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -43890,6 +44137,9 @@
       <c r="FI32">
         <v>-1.63934426229509</v>
       </c>
+      <c r="FJ32">
+        <v>-1.45278450363195</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -44387,7 +44637,10 @@
         <v>0.124533001245341</v>
       </c>
       <c r="FI33">
-        <v>-0.365408038976854</v>
+        <v>-0.121802679658946</v>
+      </c>
+      <c r="FJ33">
+        <v>-0.632911392405057</v>
       </c>
     </row>
     <row r="34">
@@ -44888,6 +45141,9 @@
       <c r="FI34">
         <v>0.260756192959586</v>
       </c>
+      <c r="FJ34">
+        <v>0.112994350282479</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -45387,6 +45643,9 @@
       <c r="FI35">
         <v>1.55763239875389</v>
       </c>
+      <c r="FJ35">
+        <v>2.57611241217797</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -45886,6 +46145,9 @@
       <c r="FI36">
         <v>0.458891013384317</v>
       </c>
+      <c r="FJ36">
+        <v>-0.729927007299274</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -46383,7 +46645,10 @@
         <v>3.36538461538462</v>
       </c>
       <c r="FI37">
-        <v>5.09193776520508</v>
+        <v>4.24328147100424</v>
+      </c>
+      <c r="FJ37">
+        <v>3.8659793814433</v>
       </c>
     </row>
     <row r="38">
@@ -46882,7 +47147,10 @@
         <v>2.7552101730837</v>
       </c>
       <c r="FI38">
-        <v>2.84589224986576</v>
+        <v>1.36030069804903</v>
+      </c>
+      <c r="FJ38">
+        <v>-0.195165891007349</v>
       </c>
     </row>
     <row r="39">
@@ -47383,6 +47651,9 @@
       <c r="FI39">
         <v>0.0649983750406203</v>
       </c>
+      <c r="FJ39">
+        <v>0.118659151587059</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -47882,6 +48153,9 @@
       <c r="FI40">
         <v>0</v>
       </c>
+      <c r="FJ40">
+        <v>-1.03092783505154</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -48379,7 +48653,10 @@
         <v>-0.514432695055717</v>
       </c>
       <c r="FI41">
-        <v>0.113314447592062</v>
+        <v>0.481586402266302</v>
+      </c>
+      <c r="FJ41">
+        <v>0.0781657113079907</v>
       </c>
     </row>
     <row r="42">
@@ -48880,6 +49157,9 @@
       <c r="FI42">
         <v>1.46520146520147</v>
       </c>
+      <c r="FJ42">
+        <v>1.62232316677482</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -49377,7 +49657,10 @@
         <v>-2.4793388429752</v>
       </c>
       <c r="FI43">
-        <v>-2.60323159784559</v>
+        <v>-1.61579892280072</v>
+      </c>
+      <c r="FJ43">
+        <v>-1.95465207193119</v>
       </c>
     </row>
     <row r="44">
@@ -49878,6 +50161,9 @@
       <c r="FI44">
         <v>0.702000702000702</v>
       </c>
+      <c r="FJ44">
+        <v>0.361336946702814</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -50377,6 +50663,9 @@
       <c r="FI45">
         <v>-1.7391304347826</v>
       </c>
+      <c r="FJ45">
+        <v>-0.344827586206889</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -50874,7 +51163,10 @@
         <v>0.952986022871683</v>
       </c>
       <c r="FI46">
-        <v>-1.08173076923078</v>
+        <v>-0.961538461538458</v>
+      </c>
+      <c r="FJ46">
+        <v>-1.01983002832862</v>
       </c>
     </row>
     <row r="47">
@@ -51375,6 +51667,9 @@
       <c r="FI47">
         <v>-1.00671140939598</v>
       </c>
+      <c r="FJ47">
+        <v>-1.05820105820105</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -51874,6 +52169,9 @@
       <c r="FI48">
         <v>2.28116710875332</v>
       </c>
+      <c r="FJ48">
+        <v>2.37319683573755</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -52371,7 +52669,10 @@
         <v>0.156971375807945</v>
       </c>
       <c r="FI49">
-        <v>0.585955106824123</v>
+        <v>0.910484089065189</v>
+      </c>
+      <c r="FJ49">
+        <v>-0.735480598529043</v>
       </c>
     </row>
     <row r="50">
@@ -52872,6 +53173,9 @@
       <c r="FI50">
         <v>-1.56249999999999</v>
       </c>
+      <c r="FJ50">
+        <v>-0.904977375565602</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -53369,7 +53673,10 @@
         <v>7.49999999999999</v>
       </c>
       <c r="FI51">
-        <v>-3.47490347490347</v>
+        <v>-2.7027027027027</v>
+      </c>
+      <c r="FJ51">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -53868,7 +54175,10 @@
         <v>1.93943518203472</v>
       </c>
       <c r="FI52">
-        <v>1.84757505773671</v>
+        <v>2.77136258660507</v>
+      </c>
+      <c r="FJ52">
+        <v>2.64251781472685</v>
       </c>
     </row>
     <row r="53">
@@ -54367,7 +54677,10 @@
         <v>-2.99057763211798</v>
       </c>
       <c r="FI53">
-        <v>-2.24331320103538</v>
+        <v>-2.41587575496117</v>
+      </c>
+      <c r="FJ53">
+        <v>-3.27537403962799</v>
       </c>
     </row>
     <row r="54">
@@ -54868,6 +55181,9 @@
       <c r="FI54">
         <v>2.75735294117647</v>
       </c>
+      <c r="FJ54">
+        <v>1.81518151815183</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -55365,7 +55681,10 @@
         <v>-1.27462340672075</v>
       </c>
       <c r="FI55">
-        <v>-3.77142857142858</v>
+        <v>-2.91428571428571</v>
+      </c>
+      <c r="FJ55">
+        <v>-2.00685266764563</v>
       </c>
     </row>
     <row r="56">
@@ -55864,7 +56183,10 @@
         <v>-4.31372549019608</v>
       </c>
       <c r="FI56">
-        <v>-3.48837209302325</v>
+        <v>-3.10077519379844</v>
+      </c>
+      <c r="FJ56">
+        <v>-0.999999999999991</v>
       </c>
     </row>
   </sheetData>

</xml_diff>